<commit_message>
Pipeline: scrape legacy + contrôle croisé (12Z)
</commit_message>
<xml_diff>
--- a/Forecasts/Forecast-02072026-12Z.xlsx
+++ b/Forecasts/Forecast-02072026-12Z.xlsx
@@ -653,7 +653,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Généré le : 02/07/2026 21:56</t>
+          <t>Généré le : 02/07/2026 22:56</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1790,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Généré le : 02/07/2026 21:56</t>
+          <t>Généré le : 02/07/2026 22:56</t>
         </is>
       </c>
     </row>

</xml_diff>